<commit_message>
Full pipeline re-run: all 8 mAbs, monkey + human, Adalimumab IV included
Script 01: regenerated configs with Adalimumab IV (5 human doses: 0.5-10 mpk)
Script 02: 43 simulation scenarios (14 monkey + 24 human + 5 Adalimumab human)
Script 03: updated plots and fold-error tables for all drugs both species

Results: SimulationResults/2026-06-18 11-23/ (43 CSVs)
Figures: 8 PK plots + PK_Metrics_ObsPred.xlsx refreshed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test2/03_Apriori/V2/Configurations/ModelParameters.xlsx
+++ b/Test2/03_Apriori/V2/Configurations/ModelParameters.xlsx
@@ -7,21 +7,22 @@
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Adalimumab_Monkey" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Atezolizumab_Human" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Atezolizumab_Monkey" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Avelumab_Human" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Avelumab_Monkey" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Bevacizumab_Human" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Bevacizumab_Monkey" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Golimumab_Human" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Golimumab_Monkey" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Nivolumab_Human" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Nivolumab_Monkey" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Pembrolizumab_Human" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Pembrolizumab_Monkey" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Tocilizumab_Human" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Tocilizumab_Monkey" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Adalimumab_Human" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Adalimumab_Monkey" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Atezolizumab_Human" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Atezolizumab_Monkey" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Avelumab_Human" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Avelumab_Monkey" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Bevacizumab_Human" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Bevacizumab_Monkey" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Golimumab_Human" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Golimumab_Monkey" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Nivolumab_Human" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Nivolumab_Monkey" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Pembrolizumab_Human" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Pembrolizumab_Monkey" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Tocilizumab_Human" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Tocilizumab_Monkey" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
 </workbook>
 </file>
@@ -600,7 +601,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00145</v>
+        <v>0.000018</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -614,7 +615,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.114</v>
+        <v>0.005583</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -628,7 +629,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>0.027</v>
+        <v>0.866</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -642,7 +643,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>0.027</v>
+        <v>0.223</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -656,7 +657,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>0.07138</v>
+        <v>0.001</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -771,7 +772,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0166</v>
+        <v>0.07138</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -816,7 +817,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.081</v>
+        <v>1.05</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -830,7 +831,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00031</v>
+        <v>0.00145</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -844,7 +845,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0017</v>
+        <v>0.114</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -886,7 +887,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>0.07138</v>
+        <v>0.0166</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -1001,7 +1002,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0166</v>
+        <v>0.07138</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -1046,7 +1047,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>1.05</v>
+        <v>0.081</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -1060,7 +1061,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00134</v>
+        <v>0.00031</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -1074,7 +1075,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.01284</v>
+        <v>0.0017</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1088,7 +1089,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>0.28</v>
+        <v>0.027</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -1102,7 +1103,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>0.28</v>
+        <v>0.027</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -1116,7 +1117,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>2.2</v>
+        <v>0.0166</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -1243,6 +1244,121 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="28.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="32.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.00134</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.01284</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -1391,7 +1507,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.65</v>
+        <v>1.05</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -1405,7 +1521,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.299</v>
+        <v>0.000127</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -1419,7 +1535,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.00936</v>
+        <v>0.0096</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1433,7 +1549,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>0.606</v>
+        <v>0.866</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -1447,7 +1563,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0426</v>
+        <v>0.223</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -1461,7 +1577,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>0.609</v>
+        <v>0.001</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -1621,7 +1737,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>1.05</v>
+        <v>0.65</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -1635,7 +1751,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0000467</v>
+        <v>0.299</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -1649,7 +1765,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.00174</v>
+        <v>0.00936</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1663,7 +1779,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>0.25</v>
+        <v>0.606</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -1865,7 +1981,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.000058</v>
+        <v>0.0000467</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -1879,7 +1995,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.00186</v>
+        <v>0.00174</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1893,7 +2009,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>0.48</v>
+        <v>0.25</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -1907,7 +2023,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>0.48</v>
+        <v>0.0426</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -1921,7 +2037,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>0.013</v>
+        <v>0.609</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -2095,7 +2211,7 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.000018</v>
+        <v>0.000058</v>
       </c>
       <c r="D3" t="s">
         <v>6</v>
@@ -2109,7 +2225,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.005583</v>
+        <v>0.00186</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -2123,7 +2239,7 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>0.866</v>
+        <v>0.48</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -2137,7 +2253,7 @@
         <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>0.223</v>
+        <v>0.48</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -2151,7 +2267,7 @@
         <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>0.001</v>
+        <v>0.013</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>

</xml_diff>